<commit_message>
Ignore backend leads data paths
Update gitignore and sync recent configuration/data changes, including docker redis port adjustments.
</commit_message>
<xml_diff>
--- a/backend/data/leads.xlsx
+++ b/backend/data/leads.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,7 +519,6 @@
           <t>ravi@techstartup.in</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>fintech</t>
@@ -535,14 +534,11 @@
           <t>good budget</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>AI automation, CRM</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>CONVERSION</t>
@@ -551,6 +547,47 @@
       <c r="O2" t="inlineStr">
         <is>
           <t>test-delivery-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-24 07:12:13</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HOT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>looking for my business website to be developed</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Understood! You're looking to establish or enhance</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ESCALATION</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>cea5e3b3-30d2-4d2f-b323-acb72d134af4</t>
         </is>
       </c>
     </row>

</xml_diff>